<commit_message>
﻿SM5: record Adam's answers to all five RFIs; correct panels to white
Panels/frames are white (drawing grey was shading); doc regenerated,
total unchanged at GBP18,611.95. Awaiting BSW alu requote of QT252647
to make the windows supplier-backed. Ack reply drafted.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/SM5 Wexham Bungalow - Fenster Pricing Document (house format).xlsx
+++ b/outputs/SM5 Wexham Bungalow - Fenster Pricing Document (house format).xlsx
@@ -2491,7 +2491,7 @@
       <c r="G5" s="10" t="n"/>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Alu windows = benchmark rates (no supplier quote yet); doors = Bellview 0000000475 net</t>
+          <t>Alu windows = benchmark rates pending BSW alu requote of QT252647; doors = Bellview 0000000475 net; white frames &amp; panels</t>
         </is>
       </c>
       <c r="I5" s="11" t="n"/>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C9" s="89" t="inlineStr">
         <is>
-          <t>W.01 - Alu window, TWO frames coupled (2no 1212 x 2400); fanlight + opener + grey infill panel below each frame</t>
+          <t>W.01 - Alu window, TWO frames coupled (2no 1212 x 2400); fanlight + opener + white infill panel below each frame</t>
         </is>
       </c>
       <c r="D9" s="90" t="n"/>
@@ -2993,7 +2993,7 @@
       </c>
       <c r="C14" s="95" t="inlineStr">
         <is>
-          <t>W.04 - Alu window, glazed head + grey infill panel below (1760mm)</t>
+          <t>W.04 - Alu window, glazed head + white infill panel below (1760mm)</t>
         </is>
       </c>
       <c r="D14" s="90" t="n"/>
@@ -3065,7 +3065,7 @@
       </c>
       <c r="C15" s="97" t="inlineStr">
         <is>
-          <t>W.05 - Alu window, glazed head + grey infill panel below (1760mm)</t>
+          <t>W.05 - Alu window, glazed head + white infill panel below (1760mm)</t>
         </is>
       </c>
       <c r="D15" s="90" t="n"/>

</xml_diff>